<commit_message>
Version 0.5.0 Name system fixes, and other changes
</commit_message>
<xml_diff>
--- a/docs/CodeSystem-retina-caution-cs.xlsx
+++ b/docs/CodeSystem-retina-caution-cs.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="44">
   <si>
     <t>Property</t>
   </si>
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.2.0</t>
+    <t>0.5.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -54,46 +54,49 @@
     <t>Experimental</t>
   </si>
   <si>
+    <t>false</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>2025-12-02</t>
+  </si>
+  <si>
+    <t>Publisher</t>
+  </si>
+  <si>
+    <t>DIPS AS</t>
+  </si>
+  <si>
+    <t>Contact</t>
+  </si>
+  <si>
+    <t>DIPS AS (http://dips.no/, teamsolsiden@dips.no)</t>
+  </si>
+  <si>
+    <t>Jurisdiction</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Cautions to consider when grading examinations (5000-series).</t>
+  </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>Copyright</t>
+  </si>
+  <si>
+    <t>Case Sensitive</t>
+  </si>
+  <si>
     <t>true</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>2025-11-30T22:57:21+01:00</t>
-  </si>
-  <si>
-    <t>Publisher</t>
-  </si>
-  <si>
-    <t>DIPS AS</t>
-  </si>
-  <si>
-    <t>Contact</t>
-  </si>
-  <si>
-    <t>DIPS AS (http://dips.no/, teamsolsiden@dips.no)</t>
-  </si>
-  <si>
-    <t>Jurisdiction</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Cautions to consider when grading examinations (5000-series).</t>
-  </si>
-  <si>
-    <t>Purpose</t>
-  </si>
-  <si>
-    <t>Copyright</t>
-  </si>
-  <si>
-    <t>Case Sensitive</t>
   </si>
   <si>
     <t>Value Set (all codes)</t>
@@ -395,53 +398,53 @@
         <v>26</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>13</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B16" s="2"/>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B17" s="2"/>
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B18" s="2"/>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B19" s="2"/>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B21" s="2"/>
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -456,30 +459,30 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="1">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B1" t="s" s="1">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C1" t="s" s="1">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D1" t="s" s="1">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B2" t="s" s="2">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s" s="2">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
0.8.0 Add gradable parameters and change from days to months for next examination
</commit_message>
<xml_diff>
--- a/docs/CodeSystem-retina-caution-cs.xlsx
+++ b/docs/CodeSystem-retina-caution-cs.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.7.0</t>
+    <t>0.8.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -42,7 +42,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>Retina Cautions</t>
+    <t>Retina Caution Codes</t>
   </si>
   <si>
     <t>Status</t>

</xml_diff>